<commit_message>
Sync graficos_nacionales y migracion_flujos
</commit_message>
<xml_diff>
--- a/output/graficos_nacionales/plot_nacional_e_basneta_a_2018.xlsx
+++ b/output/graficos_nacionales/plot_nacional_e_basneta_a_2018.xlsx
@@ -449,7 +449,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -462,7 +462,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Aysén</t>
+          <t>Aysen</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -495,7 +495,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -508,7 +508,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Aysén</t>
+          <t>Aysen</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -541,7 +541,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -554,7 +554,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Aysén</t>
+          <t>Aysen</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -587,7 +587,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -600,7 +600,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Aysén</t>
+          <t>Aysen</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -633,7 +633,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -646,7 +646,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Aysén</t>
+          <t>Aysen</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -679,7 +679,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -692,7 +692,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Aysén</t>
+          <t>Aysen</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -725,7 +725,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -771,7 +771,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -784,7 +784,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Aysén</t>
+          <t>Aysen</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -817,7 +817,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Aysén</t>
+          <t>Aysen</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -863,7 +863,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -909,7 +909,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -955,7 +955,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -1014,7 +1014,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Aysén</t>
+          <t>Aysen</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1047,7 +1047,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -1060,7 +1060,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Aysén</t>
+          <t>Aysen</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1093,7 +1093,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -1139,7 +1139,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -1185,7 +1185,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -1231,7 +1231,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -1244,7 +1244,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Ñuble</t>
+          <t>Nuble</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1277,7 +1277,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -1290,7 +1290,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Ñuble</t>
+          <t>Nuble</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1323,7 +1323,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -1369,7 +1369,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -1415,7 +1415,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -1428,7 +1428,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Ñuble</t>
+          <t>Nuble</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1461,7 +1461,7 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -1507,7 +1507,7 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -1520,7 +1520,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Ñuble</t>
+          <t>Nuble</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1553,7 +1553,7 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -1599,7 +1599,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -1612,7 +1612,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Ñuble</t>
+          <t>Nuble</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1645,7 +1645,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -1658,7 +1658,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Ñuble</t>
+          <t>Nuble</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1691,7 +1691,7 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -1737,7 +1737,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -1783,7 +1783,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -1829,7 +1829,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -1875,7 +1875,7 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -1921,7 +1921,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -1934,7 +1934,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Ñuble</t>
+          <t>Nuble</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1967,7 +1967,7 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -2013,7 +2013,7 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -2026,7 +2026,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Ñuble</t>
+          <t>Nuble</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -2059,7 +2059,7 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -2072,7 +2072,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Ñuble</t>
+          <t>Nuble</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -2105,7 +2105,7 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -2151,7 +2151,7 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -2197,7 +2197,7 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -2243,7 +2243,7 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -2289,7 +2289,7 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -2335,7 +2335,7 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -2381,7 +2381,7 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -2427,7 +2427,7 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -2440,7 +2440,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Valparaíso</t>
+          <t>Valparaiso</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -2473,7 +2473,7 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -2486,7 +2486,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Valparaíso</t>
+          <t>Valparaiso</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -2519,7 +2519,7 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -2532,7 +2532,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Ñuble</t>
+          <t>Nuble</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -2565,7 +2565,7 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -2578,7 +2578,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Valparaíso</t>
+          <t>Valparaiso</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -2611,7 +2611,7 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -2624,7 +2624,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Valparaíso</t>
+          <t>Valparaiso</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -2657,7 +2657,7 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -2703,7 +2703,7 @@
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -2716,7 +2716,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Valparaíso</t>
+          <t>Valparaiso</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -2749,7 +2749,7 @@
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -2795,7 +2795,7 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -2841,7 +2841,7 @@
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -2887,7 +2887,7 @@
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -2933,7 +2933,7 @@
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -2979,7 +2979,7 @@
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -3025,7 +3025,7 @@
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -3071,7 +3071,7 @@
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -3117,7 +3117,7 @@
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -3163,7 +3163,7 @@
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -3209,7 +3209,7 @@
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -3255,7 +3255,7 @@
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -3268,7 +3268,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Ñuble</t>
+          <t>Nuble</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -3301,7 +3301,7 @@
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -3314,7 +3314,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Valparaíso</t>
+          <t>Valparaiso</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -3360,7 +3360,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Valparaíso</t>
+          <t>Valparaiso</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -3393,7 +3393,7 @@
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -3439,7 +3439,7 @@
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -3485,7 +3485,7 @@
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -3498,7 +3498,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Ñuble</t>
+          <t>Nuble</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -3531,7 +3531,7 @@
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -3577,7 +3577,7 @@
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -3590,7 +3590,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Valparaíso</t>
+          <t>Valparaiso</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -3623,7 +3623,7 @@
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -3669,7 +3669,7 @@
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -3715,7 +3715,7 @@
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -3761,7 +3761,7 @@
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -3807,7 +3807,7 @@
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -3853,7 +3853,7 @@
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -3899,7 +3899,7 @@
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -3945,7 +3945,7 @@
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -3991,7 +3991,7 @@
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -4037,7 +4037,7 @@
       </c>
       <c r="J80" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -4083,7 +4083,7 @@
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -4129,7 +4129,7 @@
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -4142,7 +4142,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Valparaíso</t>
+          <t>Valparaiso</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -4175,7 +4175,7 @@
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -4221,7 +4221,7 @@
       </c>
       <c r="J84" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -4234,7 +4234,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Ñuble</t>
+          <t>Nuble</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -4267,7 +4267,7 @@
       </c>
       <c r="J85" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -4280,7 +4280,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Ñuble</t>
+          <t>Nuble</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -4313,7 +4313,7 @@
       </c>
       <c r="J86" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -4326,7 +4326,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Ñuble</t>
+          <t>Nuble</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -4359,7 +4359,7 @@
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -4372,7 +4372,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Valparaíso</t>
+          <t>Valparaiso</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -4405,7 +4405,7 @@
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -4451,7 +4451,7 @@
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -4464,7 +4464,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Valparaíso</t>
+          <t>Valparaiso</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -4497,7 +4497,7 @@
       </c>
       <c r="J90" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -4543,7 +4543,7 @@
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -4556,7 +4556,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Valparaíso</t>
+          <t>Valparaiso</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -4589,7 +4589,7 @@
       </c>
       <c r="J92" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -4602,7 +4602,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Ñuble</t>
+          <t>Nuble</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -4635,7 +4635,7 @@
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -4648,7 +4648,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Valparaíso</t>
+          <t>Valparaiso</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -4681,7 +4681,7 @@
       </c>
       <c r="J94" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -4694,7 +4694,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Ñuble</t>
+          <t>Nuble</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -4727,7 +4727,7 @@
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -4773,7 +4773,7 @@
       </c>
       <c r="J96" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -4819,7 +4819,7 @@
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -4832,7 +4832,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Valparaíso</t>
+          <t>Valparaiso</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -4865,7 +4865,7 @@
       </c>
       <c r="J98" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -4911,7 +4911,7 @@
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -4957,7 +4957,7 @@
       </c>
       <c r="J100" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -4970,7 +4970,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Valparaíso</t>
+          <t>Valparaiso</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -5003,7 +5003,7 @@
       </c>
       <c r="J101" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -5016,7 +5016,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Valparaíso</t>
+          <t>Valparaiso</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -5049,7 +5049,7 @@
       </c>
       <c r="J102" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -5095,7 +5095,7 @@
       </c>
       <c r="J103" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -5108,7 +5108,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Valparaíso</t>
+          <t>Valparaiso</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -5141,7 +5141,7 @@
       </c>
       <c r="J104" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -5187,7 +5187,7 @@
       </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -5233,7 +5233,7 @@
       </c>
       <c r="J106" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -5246,7 +5246,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Valparaíso</t>
+          <t>Valparaiso</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -5279,7 +5279,7 @@
       </c>
       <c r="J107" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -5325,7 +5325,7 @@
       </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -5338,7 +5338,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Ñuble</t>
+          <t>Nuble</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -5371,7 +5371,7 @@
       </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -5417,7 +5417,7 @@
       </c>
       <c r="J110" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -5463,7 +5463,7 @@
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -5509,7 +5509,7 @@
       </c>
       <c r="J112" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -5555,7 +5555,7 @@
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -5601,7 +5601,7 @@
       </c>
       <c r="J114" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -5647,7 +5647,7 @@
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -5693,7 +5693,7 @@
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -5739,7 +5739,7 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -5785,7 +5785,7 @@
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -5798,7 +5798,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Valparaíso</t>
+          <t>Valparaiso</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -5831,7 +5831,7 @@
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -5877,7 +5877,7 @@
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -5890,7 +5890,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Ñuble</t>
+          <t>Nuble</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -5923,7 +5923,7 @@
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -5969,7 +5969,7 @@
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -5982,7 +5982,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Valparaíso</t>
+          <t>Valparaiso</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
@@ -6015,7 +6015,7 @@
       </c>
       <c r="J123" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -6061,7 +6061,7 @@
       </c>
       <c r="J124" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -6107,7 +6107,7 @@
       </c>
       <c r="J125" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -6153,7 +6153,7 @@
       </c>
       <c r="J126" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -6166,7 +6166,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Valparaíso</t>
+          <t>Valparaiso</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
@@ -6199,7 +6199,7 @@
       </c>
       <c r="J127" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -6245,7 +6245,7 @@
       </c>
       <c r="J128" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -6258,7 +6258,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Valparaíso</t>
+          <t>Valparaiso</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
@@ -6291,7 +6291,7 @@
       </c>
       <c r="J129" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -6337,7 +6337,7 @@
       </c>
       <c r="J130" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -6383,7 +6383,7 @@
       </c>
       <c r="J131" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -6429,7 +6429,7 @@
       </c>
       <c r="J132" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -6475,7 +6475,7 @@
       </c>
       <c r="J133" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -6521,7 +6521,7 @@
       </c>
       <c r="J134" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -6567,7 +6567,7 @@
       </c>
       <c r="J135" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -6580,7 +6580,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>Ñuble</t>
+          <t>Nuble</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
@@ -6613,7 +6613,7 @@
       </c>
       <c r="J136" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -6659,7 +6659,7 @@
       </c>
       <c r="J137" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -6705,7 +6705,7 @@
       </c>
       <c r="J138" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -6751,7 +6751,7 @@
       </c>
       <c r="J139" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -6797,7 +6797,7 @@
       </c>
       <c r="J140" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -6843,7 +6843,7 @@
       </c>
       <c r="J141" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -6889,7 +6889,7 @@
       </c>
       <c r="J142" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -6935,7 +6935,7 @@
       </c>
       <c r="J143" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -6948,7 +6948,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>Valparaíso</t>
+          <t>Valparaiso</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
@@ -6981,7 +6981,7 @@
       </c>
       <c r="J144" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -7027,7 +7027,7 @@
       </c>
       <c r="J145" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -7073,7 +7073,7 @@
       </c>
       <c r="J146" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -7086,7 +7086,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>Valparaíso</t>
+          <t>Valparaiso</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
@@ -7119,7 +7119,7 @@
       </c>
       <c r="J147" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -7165,7 +7165,7 @@
       </c>
       <c r="J148" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -7211,7 +7211,7 @@
       </c>
       <c r="J149" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -7224,7 +7224,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>Valparaíso</t>
+          <t>Valparaiso</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
@@ -7257,7 +7257,7 @@
       </c>
       <c r="J150" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -7270,7 +7270,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>Valparaíso</t>
+          <t>Valparaiso</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
@@ -7303,7 +7303,7 @@
       </c>
       <c r="J151" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -7349,7 +7349,7 @@
       </c>
       <c r="J152" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -7395,7 +7395,7 @@
       </c>
       <c r="J153" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -7441,7 +7441,7 @@
       </c>
       <c r="J154" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -7487,7 +7487,7 @@
       </c>
       <c r="J155" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -7533,7 +7533,7 @@
       </c>
       <c r="J156" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -7546,7 +7546,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>Valparaíso</t>
+          <t>Valparaiso</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
@@ -7579,7 +7579,7 @@
       </c>
       <c r="J157" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -7592,7 +7592,7 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>Valparaíso</t>
+          <t>Valparaiso</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
@@ -7625,7 +7625,7 @@
       </c>
       <c r="J158" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -7638,7 +7638,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>Valparaíso</t>
+          <t>Valparaiso</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
@@ -7671,7 +7671,7 @@
       </c>
       <c r="J159" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -7717,7 +7717,7 @@
       </c>
       <c r="J160" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -7763,7 +7763,7 @@
       </c>
       <c r="J161" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -7809,7 +7809,7 @@
       </c>
       <c r="J162" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -7822,7 +7822,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>Valparaíso</t>
+          <t>Valparaiso</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
@@ -7855,7 +7855,7 @@
       </c>
       <c r="J163" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -7868,7 +7868,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>Valparaíso</t>
+          <t>Valparaiso</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
@@ -7901,7 +7901,7 @@
       </c>
       <c r="J164" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -7914,7 +7914,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>Ñuble</t>
+          <t>Nuble</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
@@ -7947,7 +7947,7 @@
       </c>
       <c r="J165" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -7993,7 +7993,7 @@
       </c>
       <c r="J166" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -8039,7 +8039,7 @@
       </c>
       <c r="J167" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -8052,7 +8052,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>Valparaíso</t>
+          <t>Valparaiso</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
@@ -8085,7 +8085,7 @@
       </c>
       <c r="J168" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -8131,7 +8131,7 @@
       </c>
       <c r="J169" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -8177,7 +8177,7 @@
       </c>
       <c r="J170" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -8223,7 +8223,7 @@
       </c>
       <c r="J171" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -8269,7 +8269,7 @@
       </c>
       <c r="J172" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -8315,7 +8315,7 @@
       </c>
       <c r="J173" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -8361,7 +8361,7 @@
       </c>
       <c r="J174" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -8374,7 +8374,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>Valparaíso</t>
+          <t>Valparaiso</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
@@ -8407,7 +8407,7 @@
       </c>
       <c r="J175" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -8420,7 +8420,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>Valparaíso</t>
+          <t>Valparaiso</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
@@ -8453,7 +8453,7 @@
       </c>
       <c r="J176" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -8466,7 +8466,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>Valparaíso</t>
+          <t>Valparaiso</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
@@ -8499,7 +8499,7 @@
       </c>
       <c r="J177" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -8545,7 +8545,7 @@
       </c>
       <c r="J178" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -8591,7 +8591,7 @@
       </c>
       <c r="J179" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -8637,7 +8637,7 @@
       </c>
       <c r="J180" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -8683,7 +8683,7 @@
       </c>
       <c r="J181" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -8729,7 +8729,7 @@
       </c>
       <c r="J182" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -8742,7 +8742,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>Valparaíso</t>
+          <t>Valparaiso</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
@@ -8775,7 +8775,7 @@
       </c>
       <c r="J183" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -8821,7 +8821,7 @@
       </c>
       <c r="J184" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -8867,7 +8867,7 @@
       </c>
       <c r="J185" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -8913,7 +8913,7 @@
       </c>
       <c r="J186" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -8959,7 +8959,7 @@
       </c>
       <c r="J187" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -9005,7 +9005,7 @@
       </c>
       <c r="J188" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -9051,7 +9051,7 @@
       </c>
       <c r="J189" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -9097,7 +9097,7 @@
       </c>
       <c r="J190" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -9143,7 +9143,7 @@
       </c>
       <c r="J191" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -9189,7 +9189,7 @@
       </c>
       <c r="J192" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -9235,7 +9235,7 @@
       </c>
       <c r="J193" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -9281,7 +9281,7 @@
       </c>
       <c r="J194" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -9327,7 +9327,7 @@
       </c>
       <c r="J195" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -9373,7 +9373,7 @@
       </c>
       <c r="J196" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -9419,7 +9419,7 @@
       </c>
       <c r="J197" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -9465,7 +9465,7 @@
       </c>
       <c r="J198" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -9511,7 +9511,7 @@
       </c>
       <c r="J199" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -9557,7 +9557,7 @@
       </c>
       <c r="J200" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -9603,7 +9603,7 @@
       </c>
       <c r="J201" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -9649,7 +9649,7 @@
       </c>
       <c r="J202" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -9695,7 +9695,7 @@
       </c>
       <c r="J203" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -9741,7 +9741,7 @@
       </c>
       <c r="J204" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -9787,7 +9787,7 @@
       </c>
       <c r="J205" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -9833,7 +9833,7 @@
       </c>
       <c r="J206" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -9879,7 +9879,7 @@
       </c>
       <c r="J207" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -9925,7 +9925,7 @@
       </c>
       <c r="J208" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -9971,7 +9971,7 @@
       </c>
       <c r="J209" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -9984,7 +9984,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>Tarapacá</t>
+          <t>Tarapaca</t>
         </is>
       </c>
       <c r="D210" t="inlineStr">
@@ -10017,7 +10017,7 @@
       </c>
       <c r="J210" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -10063,7 +10063,7 @@
       </c>
       <c r="J211" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -10109,7 +10109,7 @@
       </c>
       <c r="J212" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -10155,7 +10155,7 @@
       </c>
       <c r="J213" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -10201,7 +10201,7 @@
       </c>
       <c r="J214" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -10247,7 +10247,7 @@
       </c>
       <c r="J215" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -10260,7 +10260,7 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>Tarapacá</t>
+          <t>Tarapaca</t>
         </is>
       </c>
       <c r="D216" t="inlineStr">
@@ -10293,7 +10293,7 @@
       </c>
       <c r="J216" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -10339,7 +10339,7 @@
       </c>
       <c r="J217" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -10385,7 +10385,7 @@
       </c>
       <c r="J218" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -10398,7 +10398,7 @@
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>Tarapacá</t>
+          <t>Tarapaca</t>
         </is>
       </c>
       <c r="D219" t="inlineStr">
@@ -10431,7 +10431,7 @@
       </c>
       <c r="J219" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -10477,7 +10477,7 @@
       </c>
       <c r="J220" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -10523,7 +10523,7 @@
       </c>
       <c r="J221" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -10569,7 +10569,7 @@
       </c>
       <c r="J222" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -10582,7 +10582,7 @@
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>Tarapacá</t>
+          <t>Tarapaca</t>
         </is>
       </c>
       <c r="D223" t="inlineStr">
@@ -10615,7 +10615,7 @@
       </c>
       <c r="J223" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -10661,7 +10661,7 @@
       </c>
       <c r="J224" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -10707,7 +10707,7 @@
       </c>
       <c r="J225" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -10753,7 +10753,7 @@
       </c>
       <c r="J226" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -10766,7 +10766,7 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>Tarapacá</t>
+          <t>Tarapaca</t>
         </is>
       </c>
       <c r="D227" t="inlineStr">
@@ -10799,7 +10799,7 @@
       </c>
       <c r="J227" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -10812,7 +10812,7 @@
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>Tarapacá</t>
+          <t>Tarapaca</t>
         </is>
       </c>
       <c r="D228" t="inlineStr">
@@ -10845,7 +10845,7 @@
       </c>
       <c r="J228" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -10891,7 +10891,7 @@
       </c>
       <c r="J229" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -10904,7 +10904,7 @@
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>La Araucanía</t>
+          <t>La Araucania</t>
         </is>
       </c>
       <c r="D230" t="inlineStr">
@@ -10937,7 +10937,7 @@
       </c>
       <c r="J230" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -10950,7 +10950,7 @@
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>Biobío</t>
+          <t>Biobio</t>
         </is>
       </c>
       <c r="D231" t="inlineStr">
@@ -10983,7 +10983,7 @@
       </c>
       <c r="J231" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -10996,7 +10996,7 @@
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>Biobío</t>
+          <t>Biobio</t>
         </is>
       </c>
       <c r="D232" t="inlineStr">
@@ -11029,7 +11029,7 @@
       </c>
       <c r="J232" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -11075,7 +11075,7 @@
       </c>
       <c r="J233" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -11088,7 +11088,7 @@
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>Biobío</t>
+          <t>Biobio</t>
         </is>
       </c>
       <c r="D234" t="inlineStr">
@@ -11121,7 +11121,7 @@
       </c>
       <c r="J234" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -11167,7 +11167,7 @@
       </c>
       <c r="J235" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -11180,7 +11180,7 @@
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>Los Ríos</t>
+          <t>Los Rios</t>
         </is>
       </c>
       <c r="D236" t="inlineStr">
@@ -11213,7 +11213,7 @@
       </c>
       <c r="J236" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -11226,7 +11226,7 @@
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>La Araucanía</t>
+          <t>La Araucania</t>
         </is>
       </c>
       <c r="D237" t="inlineStr">
@@ -11259,7 +11259,7 @@
       </c>
       <c r="J237" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -11272,7 +11272,7 @@
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>Biobío</t>
+          <t>Biobio</t>
         </is>
       </c>
       <c r="D238" t="inlineStr">
@@ -11305,7 +11305,7 @@
       </c>
       <c r="J238" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -11351,7 +11351,7 @@
       </c>
       <c r="J239" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -11364,7 +11364,7 @@
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>Biobío</t>
+          <t>Biobio</t>
         </is>
       </c>
       <c r="D240" t="inlineStr">
@@ -11397,7 +11397,7 @@
       </c>
       <c r="J240" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -11410,7 +11410,7 @@
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>La Araucanía</t>
+          <t>La Araucania</t>
         </is>
       </c>
       <c r="D241" t="inlineStr">
@@ -11443,7 +11443,7 @@
       </c>
       <c r="J241" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -11489,7 +11489,7 @@
       </c>
       <c r="J242" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -11535,7 +11535,7 @@
       </c>
       <c r="J243" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -11548,7 +11548,7 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>La Araucanía</t>
+          <t>La Araucania</t>
         </is>
       </c>
       <c r="D244" t="inlineStr">
@@ -11581,7 +11581,7 @@
       </c>
       <c r="J244" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -11594,7 +11594,7 @@
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>Biobío</t>
+          <t>Biobio</t>
         </is>
       </c>
       <c r="D245" t="inlineStr">
@@ -11627,7 +11627,7 @@
       </c>
       <c r="J245" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -11673,7 +11673,7 @@
       </c>
       <c r="J246" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -11686,7 +11686,7 @@
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>Biobío</t>
+          <t>Biobio</t>
         </is>
       </c>
       <c r="D247" t="inlineStr">
@@ -11719,7 +11719,7 @@
       </c>
       <c r="J247" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -11732,7 +11732,7 @@
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>Biobío</t>
+          <t>Biobio</t>
         </is>
       </c>
       <c r="D248" t="inlineStr">
@@ -11765,7 +11765,7 @@
       </c>
       <c r="J248" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -11811,7 +11811,7 @@
       </c>
       <c r="J249" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -11824,7 +11824,7 @@
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>La Araucanía</t>
+          <t>La Araucania</t>
         </is>
       </c>
       <c r="D250" t="inlineStr">
@@ -11857,7 +11857,7 @@
       </c>
       <c r="J250" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -11870,7 +11870,7 @@
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>La Araucanía</t>
+          <t>La Araucania</t>
         </is>
       </c>
       <c r="D251" t="inlineStr">
@@ -11903,7 +11903,7 @@
       </c>
       <c r="J251" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -11916,7 +11916,7 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>Biobío</t>
+          <t>Biobio</t>
         </is>
       </c>
       <c r="D252" t="inlineStr">
@@ -11949,7 +11949,7 @@
       </c>
       <c r="J252" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -11962,7 +11962,7 @@
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>Biobío</t>
+          <t>Biobio</t>
         </is>
       </c>
       <c r="D253" t="inlineStr">
@@ -11995,7 +11995,7 @@
       </c>
       <c r="J253" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -12041,7 +12041,7 @@
       </c>
       <c r="J254" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -12054,7 +12054,7 @@
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>La Araucanía</t>
+          <t>La Araucania</t>
         </is>
       </c>
       <c r="D255" t="inlineStr">
@@ -12087,7 +12087,7 @@
       </c>
       <c r="J255" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -12133,7 +12133,7 @@
       </c>
       <c r="J256" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -12179,7 +12179,7 @@
       </c>
       <c r="J257" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -12192,7 +12192,7 @@
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>La Araucanía</t>
+          <t>La Araucania</t>
         </is>
       </c>
       <c r="D258" t="inlineStr">
@@ -12225,7 +12225,7 @@
       </c>
       <c r="J258" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -12238,7 +12238,7 @@
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>Los Ríos</t>
+          <t>Los Rios</t>
         </is>
       </c>
       <c r="D259" t="inlineStr">
@@ -12271,7 +12271,7 @@
       </c>
       <c r="J259" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -12284,7 +12284,7 @@
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>Los Ríos</t>
+          <t>Los Rios</t>
         </is>
       </c>
       <c r="D260" t="inlineStr">
@@ -12317,7 +12317,7 @@
       </c>
       <c r="J260" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -12330,7 +12330,7 @@
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>La Araucanía</t>
+          <t>La Araucania</t>
         </is>
       </c>
       <c r="D261" t="inlineStr">
@@ -12363,7 +12363,7 @@
       </c>
       <c r="J261" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -12376,7 +12376,7 @@
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>La Araucanía</t>
+          <t>La Araucania</t>
         </is>
       </c>
       <c r="D262" t="inlineStr">
@@ -12409,7 +12409,7 @@
       </c>
       <c r="J262" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -12422,7 +12422,7 @@
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>La Araucanía</t>
+          <t>La Araucania</t>
         </is>
       </c>
       <c r="D263" t="inlineStr">
@@ -12455,7 +12455,7 @@
       </c>
       <c r="J263" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -12501,7 +12501,7 @@
       </c>
       <c r="J264" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -12514,7 +12514,7 @@
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>La Araucanía</t>
+          <t>La Araucania</t>
         </is>
       </c>
       <c r="D265" t="inlineStr">
@@ -12547,7 +12547,7 @@
       </c>
       <c r="J265" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -12560,7 +12560,7 @@
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>La Araucanía</t>
+          <t>La Araucania</t>
         </is>
       </c>
       <c r="D266" t="inlineStr">
@@ -12593,7 +12593,7 @@
       </c>
       <c r="J266" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -12606,7 +12606,7 @@
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>La Araucanía</t>
+          <t>La Araucania</t>
         </is>
       </c>
       <c r="D267" t="inlineStr">
@@ -12639,7 +12639,7 @@
       </c>
       <c r="J267" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -12685,7 +12685,7 @@
       </c>
       <c r="J268" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -12698,7 +12698,7 @@
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>La Araucanía</t>
+          <t>La Araucania</t>
         </is>
       </c>
       <c r="D269" t="inlineStr">
@@ -12731,7 +12731,7 @@
       </c>
       <c r="J269" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -12744,7 +12744,7 @@
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>Biobío</t>
+          <t>Biobio</t>
         </is>
       </c>
       <c r="D270" t="inlineStr">
@@ -12777,7 +12777,7 @@
       </c>
       <c r="J270" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -12790,7 +12790,7 @@
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>Biobío</t>
+          <t>Biobio</t>
         </is>
       </c>
       <c r="D271" t="inlineStr">
@@ -12823,7 +12823,7 @@
       </c>
       <c r="J271" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -12836,7 +12836,7 @@
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>Biobío</t>
+          <t>Biobio</t>
         </is>
       </c>
       <c r="D272" t="inlineStr">
@@ -12869,7 +12869,7 @@
       </c>
       <c r="J272" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -12915,7 +12915,7 @@
       </c>
       <c r="J273" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -12961,7 +12961,7 @@
       </c>
       <c r="J274" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -12974,7 +12974,7 @@
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>La Araucanía</t>
+          <t>La Araucania</t>
         </is>
       </c>
       <c r="D275" t="inlineStr">
@@ -13007,7 +13007,7 @@
       </c>
       <c r="J275" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -13020,7 +13020,7 @@
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>La Araucanía</t>
+          <t>La Araucania</t>
         </is>
       </c>
       <c r="D276" t="inlineStr">
@@ -13053,7 +13053,7 @@
       </c>
       <c r="J276" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -13066,7 +13066,7 @@
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>Biobío</t>
+          <t>Biobio</t>
         </is>
       </c>
       <c r="D277" t="inlineStr">
@@ -13099,7 +13099,7 @@
       </c>
       <c r="J277" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -13112,7 +13112,7 @@
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>La Araucanía</t>
+          <t>La Araucania</t>
         </is>
       </c>
       <c r="D278" t="inlineStr">
@@ -13145,7 +13145,7 @@
       </c>
       <c r="J278" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -13158,7 +13158,7 @@
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>Biobío</t>
+          <t>Biobio</t>
         </is>
       </c>
       <c r="D279" t="inlineStr">
@@ -13191,7 +13191,7 @@
       </c>
       <c r="J279" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -13204,7 +13204,7 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>Biobío</t>
+          <t>Biobio</t>
         </is>
       </c>
       <c r="D280" t="inlineStr">
@@ -13237,7 +13237,7 @@
       </c>
       <c r="J280" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -13250,7 +13250,7 @@
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>Biobío</t>
+          <t>Biobio</t>
         </is>
       </c>
       <c r="D281" t="inlineStr">
@@ -13283,7 +13283,7 @@
       </c>
       <c r="J281" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -13296,7 +13296,7 @@
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>Los Ríos</t>
+          <t>Los Rios</t>
         </is>
       </c>
       <c r="D282" t="inlineStr">
@@ -13329,7 +13329,7 @@
       </c>
       <c r="J282" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -13342,7 +13342,7 @@
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>Biobío</t>
+          <t>Biobio</t>
         </is>
       </c>
       <c r="D283" t="inlineStr">
@@ -13375,7 +13375,7 @@
       </c>
       <c r="J283" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -13421,7 +13421,7 @@
       </c>
       <c r="J284" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -13467,7 +13467,7 @@
       </c>
       <c r="J285" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -13480,7 +13480,7 @@
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>Los Ríos</t>
+          <t>Los Rios</t>
         </is>
       </c>
       <c r="D286" t="inlineStr">
@@ -13513,7 +13513,7 @@
       </c>
       <c r="J286" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -13526,7 +13526,7 @@
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>Los Ríos</t>
+          <t>Los Rios</t>
         </is>
       </c>
       <c r="D287" t="inlineStr">
@@ -13559,7 +13559,7 @@
       </c>
       <c r="J287" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -13572,7 +13572,7 @@
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>Biobío</t>
+          <t>Biobio</t>
         </is>
       </c>
       <c r="D288" t="inlineStr">
@@ -13605,7 +13605,7 @@
       </c>
       <c r="J288" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -13618,7 +13618,7 @@
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>Biobío</t>
+          <t>Biobio</t>
         </is>
       </c>
       <c r="D289" t="inlineStr">
@@ -13651,7 +13651,7 @@
       </c>
       <c r="J289" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -13664,7 +13664,7 @@
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>La Araucanía</t>
+          <t>La Araucania</t>
         </is>
       </c>
       <c r="D290" t="inlineStr">
@@ -13697,7 +13697,7 @@
       </c>
       <c r="J290" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -13743,7 +13743,7 @@
       </c>
       <c r="J291" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -13756,7 +13756,7 @@
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>La Araucanía</t>
+          <t>La Araucania</t>
         </is>
       </c>
       <c r="D292" t="inlineStr">
@@ -13789,7 +13789,7 @@
       </c>
       <c r="J292" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -13802,7 +13802,7 @@
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>Los Ríos</t>
+          <t>Los Rios</t>
         </is>
       </c>
       <c r="D293" t="inlineStr">
@@ -13835,7 +13835,7 @@
       </c>
       <c r="J293" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -13848,7 +13848,7 @@
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>Biobío</t>
+          <t>Biobio</t>
         </is>
       </c>
       <c r="D294" t="inlineStr">
@@ -13881,7 +13881,7 @@
       </c>
       <c r="J294" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -13894,7 +13894,7 @@
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>La Araucanía</t>
+          <t>La Araucania</t>
         </is>
       </c>
       <c r="D295" t="inlineStr">
@@ -13927,7 +13927,7 @@
       </c>
       <c r="J295" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -13940,7 +13940,7 @@
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>Los Ríos</t>
+          <t>Los Rios</t>
         </is>
       </c>
       <c r="D296" t="inlineStr">
@@ -13973,7 +13973,7 @@
       </c>
       <c r="J296" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -13986,7 +13986,7 @@
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>Biobío</t>
+          <t>Biobio</t>
         </is>
       </c>
       <c r="D297" t="inlineStr">
@@ -14019,7 +14019,7 @@
       </c>
       <c r="J297" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -14032,7 +14032,7 @@
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>Biobío</t>
+          <t>Biobio</t>
         </is>
       </c>
       <c r="D298" t="inlineStr">
@@ -14065,7 +14065,7 @@
       </c>
       <c r="J298" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -14111,7 +14111,7 @@
       </c>
       <c r="J299" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -14157,7 +14157,7 @@
       </c>
       <c r="J300" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -14203,7 +14203,7 @@
       </c>
       <c r="J301" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -14249,7 +14249,7 @@
       </c>
       <c r="J302" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -14262,7 +14262,7 @@
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>Biobío</t>
+          <t>Biobio</t>
         </is>
       </c>
       <c r="D303" t="inlineStr">
@@ -14295,7 +14295,7 @@
       </c>
       <c r="J303" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -14308,7 +14308,7 @@
       </c>
       <c r="C304" t="inlineStr">
         <is>
-          <t>La Araucanía</t>
+          <t>La Araucania</t>
         </is>
       </c>
       <c r="D304" t="inlineStr">
@@ -14341,7 +14341,7 @@
       </c>
       <c r="J304" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -14387,7 +14387,7 @@
       </c>
       <c r="J305" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -14433,7 +14433,7 @@
       </c>
       <c r="J306" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -14479,7 +14479,7 @@
       </c>
       <c r="J307" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -14492,7 +14492,7 @@
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>La Araucanía</t>
+          <t>La Araucania</t>
         </is>
       </c>
       <c r="D308" t="inlineStr">
@@ -14525,7 +14525,7 @@
       </c>
       <c r="J308" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -14538,7 +14538,7 @@
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>Biobío</t>
+          <t>Biobio</t>
         </is>
       </c>
       <c r="D309" t="inlineStr">
@@ -14571,7 +14571,7 @@
       </c>
       <c r="J309" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -14617,7 +14617,7 @@
       </c>
       <c r="J310" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -14630,7 +14630,7 @@
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>La Araucanía</t>
+          <t>La Araucania</t>
         </is>
       </c>
       <c r="D311" t="inlineStr">
@@ -14663,7 +14663,7 @@
       </c>
       <c r="J311" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -14709,7 +14709,7 @@
       </c>
       <c r="J312" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -14722,7 +14722,7 @@
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>Biobío</t>
+          <t>Biobio</t>
         </is>
       </c>
       <c r="D313" t="inlineStr">
@@ -14755,7 +14755,7 @@
       </c>
       <c r="J313" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -14768,7 +14768,7 @@
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>Los Ríos</t>
+          <t>Los Rios</t>
         </is>
       </c>
       <c r="D314" t="inlineStr">
@@ -14801,7 +14801,7 @@
       </c>
       <c r="J314" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -14814,7 +14814,7 @@
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>Biobío</t>
+          <t>Biobio</t>
         </is>
       </c>
       <c r="D315" t="inlineStr">
@@ -14847,7 +14847,7 @@
       </c>
       <c r="J315" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -14860,7 +14860,7 @@
       </c>
       <c r="C316" t="inlineStr">
         <is>
-          <t>La Araucanía</t>
+          <t>La Araucania</t>
         </is>
       </c>
       <c r="D316" t="inlineStr">
@@ -14893,7 +14893,7 @@
       </c>
       <c r="J316" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -14906,7 +14906,7 @@
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t>La Araucanía</t>
+          <t>La Araucania</t>
         </is>
       </c>
       <c r="D317" t="inlineStr">
@@ -14939,7 +14939,7 @@
       </c>
       <c r="J317" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -14952,7 +14952,7 @@
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>Los Ríos</t>
+          <t>Los Rios</t>
         </is>
       </c>
       <c r="D318" t="inlineStr">
@@ -14985,7 +14985,7 @@
       </c>
       <c r="J318" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -14998,7 +14998,7 @@
       </c>
       <c r="C319" t="inlineStr">
         <is>
-          <t>Los Ríos</t>
+          <t>Los Rios</t>
         </is>
       </c>
       <c r="D319" t="inlineStr">
@@ -15031,7 +15031,7 @@
       </c>
       <c r="J319" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -15044,7 +15044,7 @@
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t>Los Ríos</t>
+          <t>Los Rios</t>
         </is>
       </c>
       <c r="D320" t="inlineStr">
@@ -15077,7 +15077,7 @@
       </c>
       <c r="J320" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -15090,7 +15090,7 @@
       </c>
       <c r="C321" t="inlineStr">
         <is>
-          <t>La Araucanía</t>
+          <t>La Araucania</t>
         </is>
       </c>
       <c r="D321" t="inlineStr">
@@ -15123,7 +15123,7 @@
       </c>
       <c r="J321" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -15136,7 +15136,7 @@
       </c>
       <c r="C322" t="inlineStr">
         <is>
-          <t>Biobío</t>
+          <t>Biobio</t>
         </is>
       </c>
       <c r="D322" t="inlineStr">
@@ -15169,7 +15169,7 @@
       </c>
       <c r="J322" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -15182,7 +15182,7 @@
       </c>
       <c r="C323" t="inlineStr">
         <is>
-          <t>La Araucanía</t>
+          <t>La Araucania</t>
         </is>
       </c>
       <c r="D323" t="inlineStr">
@@ -15215,7 +15215,7 @@
       </c>
       <c r="J323" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -15228,7 +15228,7 @@
       </c>
       <c r="C324" t="inlineStr">
         <is>
-          <t>Biobío</t>
+          <t>Biobio</t>
         </is>
       </c>
       <c r="D324" t="inlineStr">
@@ -15261,7 +15261,7 @@
       </c>
       <c r="J324" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -15274,7 +15274,7 @@
       </c>
       <c r="C325" t="inlineStr">
         <is>
-          <t>Biobío</t>
+          <t>Biobio</t>
         </is>
       </c>
       <c r="D325" t="inlineStr">
@@ -15307,7 +15307,7 @@
       </c>
       <c r="J325" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -15353,7 +15353,7 @@
       </c>
       <c r="J326" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -15366,7 +15366,7 @@
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t>La Araucanía</t>
+          <t>La Araucania</t>
         </is>
       </c>
       <c r="D327" t="inlineStr">
@@ -15399,7 +15399,7 @@
       </c>
       <c r="J327" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -15445,7 +15445,7 @@
       </c>
       <c r="J328" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -15458,7 +15458,7 @@
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>La Araucanía</t>
+          <t>La Araucania</t>
         </is>
       </c>
       <c r="D329" t="inlineStr">
@@ -15491,7 +15491,7 @@
       </c>
       <c r="J329" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -15537,7 +15537,7 @@
       </c>
       <c r="J330" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -15550,7 +15550,7 @@
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>Biobío</t>
+          <t>Biobio</t>
         </is>
       </c>
       <c r="D331" t="inlineStr">
@@ -15583,7 +15583,7 @@
       </c>
       <c r="J331" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -15596,7 +15596,7 @@
       </c>
       <c r="C332" t="inlineStr">
         <is>
-          <t>Biobío</t>
+          <t>Biobio</t>
         </is>
       </c>
       <c r="D332" t="inlineStr">
@@ -15629,7 +15629,7 @@
       </c>
       <c r="J332" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -15642,7 +15642,7 @@
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t>Biobío</t>
+          <t>Biobio</t>
         </is>
       </c>
       <c r="D333" t="inlineStr">
@@ -15675,7 +15675,7 @@
       </c>
       <c r="J333" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -15688,7 +15688,7 @@
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>La Araucanía</t>
+          <t>La Araucania</t>
         </is>
       </c>
       <c r="D334" t="inlineStr">
@@ -15721,7 +15721,7 @@
       </c>
       <c r="J334" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -15767,7 +15767,7 @@
       </c>
       <c r="J335" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>
@@ -15780,7 +15780,7 @@
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>La Araucanía</t>
+          <t>La Araucania</t>
         </is>
       </c>
       <c r="D336" t="inlineStr">
@@ -15813,7 +15813,7 @@
       </c>
       <c r="J336" t="inlineStr">
         <is>
-          <t>Tasa neta básica</t>
+          <t>Tasa neta basica</t>
         </is>
       </c>
     </row>

</xml_diff>